<commit_message>
fix(data): update ver4 false claim wording
</commit_message>
<xml_diff>
--- a/Ver4/testdata/エクセル/real_article_dataset_v2_reading_guide.xlsx
+++ b/Ver4/testdata/エクセル/real_article_dataset_v2_reading_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9733118985f6bf19/Desktop/datamix/講義/05_インテグレーションステップ/fake-news-checker/Ver4/testdata/エクセル/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{E542DCC9-FE14-46B2-B9A9-8DCE0AE66852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEFEE01F-EEC4-4C00-BC21-D7B9F1405C02}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{E542DCC9-FE14-46B2-B9A9-8DCE0AE66852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{625D1B57-188C-41CF-872F-4710D0C99044}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1420F31D-1235-43A3-BC87-6F880C98AB5A}"/>
   </bookViews>
@@ -672,12 +672,6 @@
     <t>朝日新聞の入社式では、社旗の脇に韓国と中国の国旗を並べ、ハングル文字を掲げていた。</t>
   </si>
   <si>
-    <t>jfc-false-15-false-100k-demo-osaka-yoon</t>
-  </si>
-  <si>
-    <t>大阪で10万人のデモ隊が韓国の尹錫悦大統領の罷免と拘束や、日本と断交し北朝鮮やロシアと国交を回復することを要求した。</t>
-  </si>
-  <si>
     <t>jfc-false-16-false-minimum-access-rice-harmful</t>
   </si>
   <si>
@@ -730,6 +724,17 @@
     <rPh sb="60" eb="61">
       <t>ナ</t>
     </rPh>
+    <phoneticPr fontId="18"/>
+  </si>
+  <si>
+    <t>大阪で在日コリアン10万人のデモ隊が日本と断交し、北朝鮮やロシアと国交を回復することを要求した。</t>
+    <rPh sb="3" eb="5">
+      <t>ザイニチ</t>
+    </rPh>
+    <phoneticPr fontId="18"/>
+  </si>
+  <si>
+    <t>jfc-false-15-false-100k-demo-osaka-yoon</t>
     <phoneticPr fontId="18"/>
   </si>
 </sst>
@@ -1709,7 +1714,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -1718,10 +1723,10 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H1" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
@@ -3463,7 +3468,7 @@
         <v>7</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E66" t="s">
         <v>142</v>
@@ -3472,7 +3477,7 @@
         <v>143</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H66" t="b">
         <f t="shared" si="0"/>
@@ -4264,7 +4269,7 @@
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="B96" t="s">
         <v>182</v>
@@ -4272,8 +4277,8 @@
       <c r="C96" t="s">
         <v>29</v>
       </c>
-      <c r="D96" t="s">
-        <v>213</v>
+      <c r="D96" s="1" t="s">
+        <v>226</v>
       </c>
       <c r="E96" t="s">
         <v>184</v>
@@ -4281,8 +4286,8 @@
       <c r="F96" t="s">
         <v>185</v>
       </c>
-      <c r="G96" t="s">
-        <v>213</v>
+      <c r="G96" s="1" t="s">
+        <v>226</v>
       </c>
       <c r="H96" t="b">
         <f t="shared" si="1"/>
@@ -4291,7 +4296,7 @@
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B97" t="s">
         <v>182</v>
@@ -4300,7 +4305,7 @@
         <v>7</v>
       </c>
       <c r="D97" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="E97" t="s">
         <v>184</v>
@@ -4309,7 +4314,7 @@
         <v>185</v>
       </c>
       <c r="G97" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="H97" t="b">
         <f t="shared" si="1"/>
@@ -4318,7 +4323,7 @@
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B98" t="s">
         <v>182</v>
@@ -4327,7 +4332,7 @@
         <v>7</v>
       </c>
       <c r="D98" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E98" t="s">
         <v>184</v>
@@ -4336,7 +4341,7 @@
         <v>185</v>
       </c>
       <c r="G98" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="H98" t="b">
         <f t="shared" si="1"/>
@@ -4345,7 +4350,7 @@
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B99" t="s">
         <v>182</v>
@@ -4354,7 +4359,7 @@
         <v>7</v>
       </c>
       <c r="D99" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E99" t="s">
         <v>184</v>
@@ -4363,7 +4368,7 @@
         <v>185</v>
       </c>
       <c r="G99" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="H99" t="b">
         <f t="shared" si="1"/>
@@ -4372,7 +4377,7 @@
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B100" t="s">
         <v>182</v>
@@ -4381,7 +4386,7 @@
         <v>7</v>
       </c>
       <c r="D100" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E100" t="s">
         <v>184</v>
@@ -4390,7 +4395,7 @@
         <v>185</v>
       </c>
       <c r="G100" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H100" t="b">
         <f t="shared" si="1"/>
@@ -4399,7 +4404,7 @@
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B101" t="s">
         <v>182</v>
@@ -4408,7 +4413,7 @@
         <v>7</v>
       </c>
       <c r="D101" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E101" t="s">
         <v>184</v>
@@ -4417,7 +4422,7 @@
         <v>185</v>
       </c>
       <c r="G101" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="H101" t="b">
         <f t="shared" si="1"/>

</xml_diff>

<commit_message>
Sync Ver2 updates into Ver3/Ver4 and tighten claim-mode verdicts
</commit_message>
<xml_diff>
--- a/Ver4/testdata/エクセル/real_article_dataset_v2_reading_guide.xlsx
+++ b/Ver4/testdata/エクセル/real_article_dataset_v2_reading_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9733118985f6bf19/Desktop/datamix/講義/05_インテグレーションステップ/fake-news-checker/Ver4/testdata/エクセル/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{E542DCC9-FE14-46B2-B9A9-8DCE0AE66852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{625D1B57-188C-41CF-872F-4710D0C99044}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{E542DCC9-FE14-46B2-B9A9-8DCE0AE66852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{065C7183-D925-449B-A633-1F741EFC7C8B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1420F31D-1235-43A3-BC87-6F880C98AB5A}"/>
   </bookViews>
@@ -477,9 +477,6 @@
     <t>jfc-inaccurate-03-japan-is-not-expanding-the-pakistani-intake-to-50thousands</t>
   </si>
   <si>
-    <t>スタジオジブリ制作のアニメ映画「となりのトトロ」と「火垂るの墓」は1988年4月に同時上映された。「となりのトトロ」は高畑勲、「火垂るの墓」は宮崎駿の監督作品で、プロデューサーは庵野秀明だった。</t>
-  </si>
-  <si>
     <t>jfc-inaccurate-04-inaccurate-kyoto-hotel-prices-collapse</t>
   </si>
   <si>
@@ -735,6 +732,10 @@
   </si>
   <si>
     <t>jfc-false-15-false-100k-demo-osaka-yoon</t>
+    <phoneticPr fontId="18"/>
+  </si>
+  <si>
+    <t>スタジオジブリ制作のアニメ映画「となりのトトロ」と「火垂るの墓」は1988年4月に同時上映された。「となりのトトロ」は高畑勲、「火垂るの墓」は宮崎駿の監督作品である。</t>
     <phoneticPr fontId="18"/>
   </si>
 </sst>
@@ -1714,7 +1715,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -1723,10 +1724,10 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
@@ -3413,8 +3414,8 @@
       <c r="C64" t="s">
         <v>7</v>
       </c>
-      <c r="D64" t="s">
-        <v>147</v>
+      <c r="D64" s="1" t="s">
+        <v>227</v>
       </c>
       <c r="E64" t="s">
         <v>142</v>
@@ -3422,8 +3423,8 @@
       <c r="F64" t="s">
         <v>143</v>
       </c>
-      <c r="G64" t="s">
-        <v>147</v>
+      <c r="G64" s="1" t="s">
+        <v>227</v>
       </c>
       <c r="H64" t="b">
         <f t="shared" si="0"/>
@@ -3432,7 +3433,7 @@
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B65" t="s">
         <v>140</v>
@@ -3441,7 +3442,7 @@
         <v>7</v>
       </c>
       <c r="D65" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E65" t="s">
         <v>142</v>
@@ -3450,7 +3451,7 @@
         <v>143</v>
       </c>
       <c r="G65" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H65" t="b">
         <f t="shared" si="0"/>
@@ -3459,7 +3460,7 @@
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B66" t="s">
         <v>140</v>
@@ -3468,7 +3469,7 @@
         <v>7</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E66" t="s">
         <v>142</v>
@@ -3477,7 +3478,7 @@
         <v>143</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H66" t="b">
         <f t="shared" si="0"/>
@@ -3486,7 +3487,7 @@
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B67" t="s">
         <v>140</v>
@@ -3495,7 +3496,7 @@
         <v>7</v>
       </c>
       <c r="D67" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E67" t="s">
         <v>142</v>
@@ -3504,7 +3505,7 @@
         <v>143</v>
       </c>
       <c r="G67" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H67" t="b">
         <f t="shared" ref="H67:H101" si="1">EXACT(D67,G67)</f>
@@ -3513,7 +3514,7 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B68" t="s">
         <v>140</v>
@@ -3522,7 +3523,7 @@
         <v>7</v>
       </c>
       <c r="D68" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E68" t="s">
         <v>142</v>
@@ -3531,7 +3532,7 @@
         <v>143</v>
       </c>
       <c r="G68" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H68" t="b">
         <f t="shared" si="1"/>
@@ -3540,7 +3541,7 @@
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B69" t="s">
         <v>140</v>
@@ -3549,7 +3550,7 @@
         <v>7</v>
       </c>
       <c r="D69" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E69" t="s">
         <v>142</v>
@@ -3558,7 +3559,7 @@
         <v>143</v>
       </c>
       <c r="G69" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H69" t="b">
         <f t="shared" si="1"/>
@@ -3567,7 +3568,7 @@
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B70" t="s">
         <v>140</v>
@@ -3576,7 +3577,7 @@
         <v>7</v>
       </c>
       <c r="D70" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E70" t="s">
         <v>142</v>
@@ -3585,7 +3586,7 @@
         <v>143</v>
       </c>
       <c r="G70" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H70" t="b">
         <f t="shared" si="1"/>
@@ -3594,7 +3595,7 @@
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B71" t="s">
         <v>140</v>
@@ -3603,7 +3604,7 @@
         <v>7</v>
       </c>
       <c r="D71" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E71" t="s">
         <v>142</v>
@@ -3612,7 +3613,7 @@
         <v>143</v>
       </c>
       <c r="G71" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H71" t="b">
         <f t="shared" si="1"/>
@@ -3621,7 +3622,7 @@
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B72" t="s">
         <v>140</v>
@@ -3630,7 +3631,7 @@
         <v>29</v>
       </c>
       <c r="D72" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E72" t="s">
         <v>142</v>
@@ -3639,7 +3640,7 @@
         <v>143</v>
       </c>
       <c r="G72" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H72" t="b">
         <f t="shared" si="1"/>
@@ -3648,7 +3649,7 @@
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B73" t="s">
         <v>140</v>
@@ -3657,7 +3658,7 @@
         <v>7</v>
       </c>
       <c r="D73" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E73" t="s">
         <v>142</v>
@@ -3666,7 +3667,7 @@
         <v>143</v>
       </c>
       <c r="G73" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H73" t="b">
         <f t="shared" si="1"/>
@@ -3675,7 +3676,7 @@
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B74" t="s">
         <v>140</v>
@@ -3684,7 +3685,7 @@
         <v>7</v>
       </c>
       <c r="D74" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E74" t="s">
         <v>142</v>
@@ -3693,7 +3694,7 @@
         <v>143</v>
       </c>
       <c r="G74" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H74" t="b">
         <f t="shared" si="1"/>
@@ -3702,7 +3703,7 @@
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B75" t="s">
         <v>140</v>
@@ -3711,7 +3712,7 @@
         <v>7</v>
       </c>
       <c r="D75" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E75" t="s">
         <v>142</v>
@@ -3720,7 +3721,7 @@
         <v>143</v>
       </c>
       <c r="G75" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H75" t="b">
         <f t="shared" si="1"/>
@@ -3729,7 +3730,7 @@
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B76" t="s">
         <v>140</v>
@@ -3738,7 +3739,7 @@
         <v>7</v>
       </c>
       <c r="D76" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E76" t="s">
         <v>142</v>
@@ -3747,7 +3748,7 @@
         <v>143</v>
       </c>
       <c r="G76" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H76" t="b">
         <f t="shared" si="1"/>
@@ -3756,7 +3757,7 @@
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B77" t="s">
         <v>140</v>
@@ -3765,7 +3766,7 @@
         <v>7</v>
       </c>
       <c r="D77" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E77" t="s">
         <v>142</v>
@@ -3774,7 +3775,7 @@
         <v>143</v>
       </c>
       <c r="G77" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H77" t="b">
         <f t="shared" si="1"/>
@@ -3783,7 +3784,7 @@
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B78" t="s">
         <v>140</v>
@@ -3792,7 +3793,7 @@
         <v>7</v>
       </c>
       <c r="D78" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E78" t="s">
         <v>142</v>
@@ -3801,7 +3802,7 @@
         <v>143</v>
       </c>
       <c r="G78" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H78" t="b">
         <f t="shared" si="1"/>
@@ -3810,7 +3811,7 @@
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B79" t="s">
         <v>140</v>
@@ -3819,7 +3820,7 @@
         <v>7</v>
       </c>
       <c r="D79" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E79" t="s">
         <v>142</v>
@@ -3828,7 +3829,7 @@
         <v>143</v>
       </c>
       <c r="G79" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H79" t="b">
         <f t="shared" si="1"/>
@@ -3837,7 +3838,7 @@
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B80" t="s">
         <v>140</v>
@@ -3846,7 +3847,7 @@
         <v>29</v>
       </c>
       <c r="D80" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E80" t="s">
         <v>142</v>
@@ -3855,7 +3856,7 @@
         <v>143</v>
       </c>
       <c r="G80" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H80" t="b">
         <f t="shared" si="1"/>
@@ -3864,7 +3865,7 @@
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B81" t="s">
         <v>140</v>
@@ -3873,7 +3874,7 @@
         <v>29</v>
       </c>
       <c r="D81" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E81" t="s">
         <v>142</v>
@@ -3882,7 +3883,7 @@
         <v>143</v>
       </c>
       <c r="G81" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H81" t="b">
         <f t="shared" si="1"/>
@@ -3891,25 +3892,25 @@
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
+        <v>180</v>
+      </c>
+      <c r="B82" t="s">
         <v>181</v>
-      </c>
-      <c r="B82" t="s">
-        <v>182</v>
       </c>
       <c r="C82" t="s">
         <v>29</v>
       </c>
       <c r="D82" t="s">
+        <v>182</v>
+      </c>
+      <c r="E82" t="s">
         <v>183</v>
       </c>
-      <c r="E82" t="s">
+      <c r="F82" t="s">
         <v>184</v>
       </c>
-      <c r="F82" t="s">
-        <v>185</v>
-      </c>
       <c r="G82" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H82" t="b">
         <f t="shared" si="1"/>
@@ -3918,25 +3919,25 @@
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
+        <v>185</v>
+      </c>
+      <c r="B83" t="s">
+        <v>181</v>
+      </c>
+      <c r="C83" t="s">
+        <v>7</v>
+      </c>
+      <c r="D83" t="s">
         <v>186</v>
       </c>
-      <c r="B83" t="s">
-        <v>182</v>
-      </c>
-      <c r="C83" t="s">
-        <v>7</v>
-      </c>
-      <c r="D83" t="s">
-        <v>187</v>
-      </c>
       <c r="E83" t="s">
+        <v>183</v>
+      </c>
+      <c r="F83" t="s">
         <v>184</v>
       </c>
-      <c r="F83" t="s">
-        <v>185</v>
-      </c>
       <c r="G83" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H83" t="b">
         <f t="shared" si="1"/>
@@ -3945,25 +3946,25 @@
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
+        <v>187</v>
+      </c>
+      <c r="B84" t="s">
+        <v>181</v>
+      </c>
+      <c r="C84" t="s">
+        <v>7</v>
+      </c>
+      <c r="D84" t="s">
         <v>188</v>
       </c>
-      <c r="B84" t="s">
-        <v>182</v>
-      </c>
-      <c r="C84" t="s">
-        <v>7</v>
-      </c>
-      <c r="D84" t="s">
-        <v>189</v>
-      </c>
       <c r="E84" t="s">
+        <v>183</v>
+      </c>
+      <c r="F84" t="s">
         <v>184</v>
       </c>
-      <c r="F84" t="s">
-        <v>185</v>
-      </c>
       <c r="G84" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="H84" t="b">
         <f t="shared" si="1"/>
@@ -3972,25 +3973,25 @@
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B85" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C85" t="s">
         <v>16</v>
       </c>
       <c r="D85" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E85" t="s">
+        <v>183</v>
+      </c>
+      <c r="F85" t="s">
         <v>184</v>
       </c>
-      <c r="F85" t="s">
-        <v>185</v>
-      </c>
       <c r="G85" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H85" t="b">
         <f t="shared" si="1"/>
@@ -3999,25 +4000,25 @@
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
+        <v>191</v>
+      </c>
+      <c r="B86" t="s">
+        <v>181</v>
+      </c>
+      <c r="C86" t="s">
+        <v>7</v>
+      </c>
+      <c r="D86" t="s">
         <v>192</v>
       </c>
-      <c r="B86" t="s">
-        <v>182</v>
-      </c>
-      <c r="C86" t="s">
-        <v>7</v>
-      </c>
-      <c r="D86" t="s">
-        <v>193</v>
-      </c>
       <c r="E86" t="s">
+        <v>183</v>
+      </c>
+      <c r="F86" t="s">
         <v>184</v>
       </c>
-      <c r="F86" t="s">
-        <v>185</v>
-      </c>
       <c r="G86" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H86" t="b">
         <f t="shared" si="1"/>
@@ -4026,25 +4027,25 @@
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B87" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C87" t="s">
         <v>16</v>
       </c>
       <c r="D87" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E87" t="s">
+        <v>183</v>
+      </c>
+      <c r="F87" t="s">
         <v>184</v>
       </c>
-      <c r="F87" t="s">
-        <v>185</v>
-      </c>
       <c r="G87" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H87" t="b">
         <f t="shared" si="1"/>
@@ -4053,25 +4054,25 @@
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B88" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C88" t="s">
         <v>123</v>
       </c>
       <c r="D88" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E88" t="s">
+        <v>183</v>
+      </c>
+      <c r="F88" t="s">
         <v>184</v>
       </c>
-      <c r="F88" t="s">
-        <v>185</v>
-      </c>
       <c r="G88" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H88" t="b">
         <f t="shared" si="1"/>
@@ -4080,25 +4081,25 @@
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
+        <v>197</v>
+      </c>
+      <c r="B89" t="s">
+        <v>181</v>
+      </c>
+      <c r="C89" t="s">
+        <v>7</v>
+      </c>
+      <c r="D89" t="s">
         <v>198</v>
       </c>
-      <c r="B89" t="s">
-        <v>182</v>
-      </c>
-      <c r="C89" t="s">
-        <v>7</v>
-      </c>
-      <c r="D89" t="s">
-        <v>199</v>
-      </c>
       <c r="E89" t="s">
+        <v>183</v>
+      </c>
+      <c r="F89" t="s">
         <v>184</v>
       </c>
-      <c r="F89" t="s">
-        <v>185</v>
-      </c>
       <c r="G89" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H89" t="b">
         <f t="shared" si="1"/>
@@ -4107,25 +4108,25 @@
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B90" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C90" t="s">
         <v>16</v>
       </c>
       <c r="D90" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E90" t="s">
+        <v>183</v>
+      </c>
+      <c r="F90" t="s">
         <v>184</v>
       </c>
-      <c r="F90" t="s">
-        <v>185</v>
-      </c>
       <c r="G90" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H90" t="b">
         <f t="shared" si="1"/>
@@ -4134,25 +4135,25 @@
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B91" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C91" t="s">
         <v>29</v>
       </c>
       <c r="D91" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E91" t="s">
+        <v>183</v>
+      </c>
+      <c r="F91" t="s">
         <v>184</v>
       </c>
-      <c r="F91" t="s">
-        <v>185</v>
-      </c>
       <c r="G91" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H91" t="b">
         <f t="shared" si="1"/>
@@ -4161,25 +4162,25 @@
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
+        <v>203</v>
+      </c>
+      <c r="B92" t="s">
+        <v>181</v>
+      </c>
+      <c r="C92" t="s">
+        <v>7</v>
+      </c>
+      <c r="D92" t="s">
         <v>204</v>
       </c>
-      <c r="B92" t="s">
-        <v>182</v>
-      </c>
-      <c r="C92" t="s">
-        <v>7</v>
-      </c>
-      <c r="D92" t="s">
-        <v>205</v>
-      </c>
       <c r="E92" t="s">
+        <v>183</v>
+      </c>
+      <c r="F92" t="s">
         <v>184</v>
       </c>
-      <c r="F92" t="s">
-        <v>185</v>
-      </c>
       <c r="G92" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H92" t="b">
         <f t="shared" si="1"/>
@@ -4188,25 +4189,25 @@
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
+        <v>205</v>
+      </c>
+      <c r="B93" t="s">
+        <v>181</v>
+      </c>
+      <c r="C93" t="s">
+        <v>7</v>
+      </c>
+      <c r="D93" t="s">
         <v>206</v>
       </c>
-      <c r="B93" t="s">
-        <v>182</v>
-      </c>
-      <c r="C93" t="s">
-        <v>7</v>
-      </c>
-      <c r="D93" t="s">
-        <v>207</v>
-      </c>
       <c r="E93" t="s">
+        <v>183</v>
+      </c>
+      <c r="F93" t="s">
         <v>184</v>
       </c>
-      <c r="F93" t="s">
-        <v>185</v>
-      </c>
       <c r="G93" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H93" t="b">
         <f t="shared" si="1"/>
@@ -4215,25 +4216,25 @@
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B94" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C94" t="s">
         <v>29</v>
       </c>
       <c r="D94" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E94" t="s">
+        <v>183</v>
+      </c>
+      <c r="F94" t="s">
         <v>184</v>
       </c>
-      <c r="F94" t="s">
-        <v>185</v>
-      </c>
       <c r="G94" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H94" t="b">
         <f t="shared" si="1"/>
@@ -4242,25 +4243,25 @@
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
+        <v>209</v>
+      </c>
+      <c r="B95" t="s">
+        <v>181</v>
+      </c>
+      <c r="C95" t="s">
+        <v>7</v>
+      </c>
+      <c r="D95" t="s">
         <v>210</v>
       </c>
-      <c r="B95" t="s">
-        <v>182</v>
-      </c>
-      <c r="C95" t="s">
-        <v>7</v>
-      </c>
-      <c r="D95" t="s">
-        <v>211</v>
-      </c>
       <c r="E95" t="s">
+        <v>183</v>
+      </c>
+      <c r="F95" t="s">
         <v>184</v>
       </c>
-      <c r="F95" t="s">
-        <v>185</v>
-      </c>
       <c r="G95" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H95" t="b">
         <f t="shared" si="1"/>
@@ -4269,25 +4270,25 @@
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B96" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C96" t="s">
         <v>29</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E96" t="s">
+        <v>183</v>
+      </c>
+      <c r="F96" t="s">
         <v>184</v>
       </c>
-      <c r="F96" t="s">
-        <v>185</v>
-      </c>
       <c r="G96" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H96" t="b">
         <f t="shared" si="1"/>
@@ -4296,25 +4297,25 @@
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
+        <v>211</v>
+      </c>
+      <c r="B97" t="s">
+        <v>181</v>
+      </c>
+      <c r="C97" t="s">
+        <v>7</v>
+      </c>
+      <c r="D97" t="s">
         <v>212</v>
       </c>
-      <c r="B97" t="s">
-        <v>182</v>
-      </c>
-      <c r="C97" t="s">
-        <v>7</v>
-      </c>
-      <c r="D97" t="s">
-        <v>213</v>
-      </c>
       <c r="E97" t="s">
+        <v>183</v>
+      </c>
+      <c r="F97" t="s">
         <v>184</v>
       </c>
-      <c r="F97" t="s">
-        <v>185</v>
-      </c>
       <c r="G97" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H97" t="b">
         <f t="shared" si="1"/>
@@ -4323,25 +4324,25 @@
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
+        <v>213</v>
+      </c>
+      <c r="B98" t="s">
+        <v>181</v>
+      </c>
+      <c r="C98" t="s">
+        <v>7</v>
+      </c>
+      <c r="D98" t="s">
         <v>214</v>
       </c>
-      <c r="B98" t="s">
-        <v>182</v>
-      </c>
-      <c r="C98" t="s">
-        <v>7</v>
-      </c>
-      <c r="D98" t="s">
-        <v>215</v>
-      </c>
       <c r="E98" t="s">
+        <v>183</v>
+      </c>
+      <c r="F98" t="s">
         <v>184</v>
       </c>
-      <c r="F98" t="s">
-        <v>185</v>
-      </c>
       <c r="G98" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H98" t="b">
         <f t="shared" si="1"/>
@@ -4350,25 +4351,25 @@
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
+        <v>215</v>
+      </c>
+      <c r="B99" t="s">
+        <v>181</v>
+      </c>
+      <c r="C99" t="s">
+        <v>7</v>
+      </c>
+      <c r="D99" t="s">
         <v>216</v>
       </c>
-      <c r="B99" t="s">
-        <v>182</v>
-      </c>
-      <c r="C99" t="s">
-        <v>7</v>
-      </c>
-      <c r="D99" t="s">
-        <v>217</v>
-      </c>
       <c r="E99" t="s">
+        <v>183</v>
+      </c>
+      <c r="F99" t="s">
         <v>184</v>
       </c>
-      <c r="F99" t="s">
-        <v>185</v>
-      </c>
       <c r="G99" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H99" t="b">
         <f t="shared" si="1"/>
@@ -4377,25 +4378,25 @@
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
+        <v>217</v>
+      </c>
+      <c r="B100" t="s">
+        <v>181</v>
+      </c>
+      <c r="C100" t="s">
+        <v>7</v>
+      </c>
+      <c r="D100" t="s">
         <v>218</v>
       </c>
-      <c r="B100" t="s">
-        <v>182</v>
-      </c>
-      <c r="C100" t="s">
-        <v>7</v>
-      </c>
-      <c r="D100" t="s">
-        <v>219</v>
-      </c>
       <c r="E100" t="s">
+        <v>183</v>
+      </c>
+      <c r="F100" t="s">
         <v>184</v>
       </c>
-      <c r="F100" t="s">
-        <v>185</v>
-      </c>
       <c r="G100" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H100" t="b">
         <f t="shared" si="1"/>
@@ -4404,25 +4405,25 @@
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
+        <v>219</v>
+      </c>
+      <c r="B101" t="s">
+        <v>181</v>
+      </c>
+      <c r="C101" t="s">
+        <v>7</v>
+      </c>
+      <c r="D101" t="s">
         <v>220</v>
       </c>
-      <c r="B101" t="s">
-        <v>182</v>
-      </c>
-      <c r="C101" t="s">
-        <v>7</v>
-      </c>
-      <c r="D101" t="s">
-        <v>221</v>
-      </c>
       <c r="E101" t="s">
+        <v>183</v>
+      </c>
+      <c r="F101" t="s">
         <v>184</v>
       </c>
-      <c r="F101" t="s">
-        <v>185</v>
-      </c>
       <c r="G101" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H101" t="b">
         <f t="shared" si="1"/>

</xml_diff>